<commit_message>
Switch to Mac Mail app for university Outlook, follow up after 7 days
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VCCszvanoGx6xKsUuBayQM
</commit_message>
<xml_diff>
--- a/outreach_template.xlsx
+++ b/outreach_template.xlsx
@@ -661,21 +661,21 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Delivery    'Delivered to server', 'Bounced', 'Failed: ...', or 'Waiting: fill in ...' if a field is missing</t>
+          <t xml:space="preserve">     Delivery    'Sent', 'Bounced', 'Failed: ...', or 'Waiting: fill in ...' if a field is missing</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Replied     Yes / No - checked against your inbox every run</t>
+          <t xml:space="preserve">     Replied     Yes / No - checked against your inbox (Mail app) every run</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Follow Up   the date the follow-up was sent (only if they haven't replied after the configured # of workdays)</t>
+          <t xml:space="preserve">     Follow Up   the date the follow-up was sent (only if they haven't replied within 7 days)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SNHU email templates; Commonality column picks which template is sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VCCszvanoGx6xKsUuBayQM
</commit_message>
<xml_diff>
--- a/outreach_template.xlsx
+++ b/outreach_template.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -626,85 +626,92 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Last Name, Company Name and Role are optional (only needed if your email draft uses them).</t>
+          <t xml:space="preserve">   Commonality picks the email template: type SNHU to send the SNHU email.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2. Leave Status EMPTY for new people. Empty Status = 'send the first email at the next 11:00 AM weekday run'.</t>
+          <t xml:space="preserve">   Last Name, Company Name and Role are optional.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3. The GREY columns are filled in automatically - don't type in them:</t>
+          <t>2. Leave Status EMPTY for new people. Empty Status = 'send the first email at the next 11:00 AM weekday run'.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Status      Sent -&gt; Followed Up -&gt; Replied   (or Bounced / Failed)</t>
+          <t>3. The GREY columns are filled in automatically - don't type in them:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Date Sent   the day the first email went out</t>
+          <t xml:space="preserve">     Status      Sent -&gt; Followed Up -&gt; Replied   (or Bounced / Failed)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Delivery    'Sent', 'Bounced', 'Failed: ...', or 'Waiting: fill in ...' if a field is missing</t>
+          <t xml:space="preserve">     Date Sent   the day the first email went out</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Replied     Yes / No - checked against your inbox (Mail app) every run</t>
+          <t xml:space="preserve">     Delivery    'Sent', 'Bounced', 'Failed: ...', or 'Waiting: fill in ...' if a field is missing</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Follow Up   the date the follow-up was sent (only if they haven't replied within 7 days)</t>
+          <t xml:space="preserve">     Replied     Yes / No - checked against your inbox (Mail app) every run</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>4. To stop emailing someone, set their Status to 'Do Not Contact'. If they replied outside email, set Replied = Yes.</t>
+          <t xml:space="preserve">     Follow Up   the date the follow-up was sent (only if they haven't replied within 7 days)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>5. CLOSE this file in Excel before 11:00 AM so the script can save its updates.</t>
+          <t>4. To stop emailing someone, set their Status to 'Do Not Contact'. If they replied outside email, set Replied = Yes.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>5. CLOSE this file in Excel before 11:00 AM so the script can save its updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">   (If it's open, the script saves a copy called outreach_UPDATED_&lt;date&gt;.xlsx instead.)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Row colours: blue = sent, yellow = followed up, green = replied, red = bounced/failed.</t>
         </is>

</xml_diff>